<commit_message>
data: Actualización automática de reportes (2026-04-13 12:03)
</commit_message>
<xml_diff>
--- a/administrador/directorio_asesores.xlsx
+++ b/administrador/directorio_asesores.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B423274E-8717-E641-93F5-8BDA340203C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A907013C-2105-D742-A17A-34758C720AC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
   <si>
     <t>Clave</t>
   </si>
@@ -192,19 +192,34 @@
   </si>
   <si>
     <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
+  </si>
+  <si>
+    <t>PAULA ANGELICA LOMELI CAZARES</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -227,8 +242,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -568,7 +585,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B52"/>
+  <dimension ref="A1:B53"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -985,6 +1002,14 @@
       </c>
       <c r="B52" t="s">
         <v>52</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A53" s="2">
+        <v>116876</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-04-15 12:36)
</commit_message>
<xml_diff>
--- a/administrador/directorio_asesores.xlsx
+++ b/administrador/directorio_asesores.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B906CED-194C-DD49-B970-2A9BECB5ABA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02F7E6AB-177F-F349-97C0-2F6D0D2240A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="55">
   <si>
     <t>Clave</t>
   </si>
@@ -195,13 +195,16 @@
   </si>
   <si>
     <t>PAULA ANGELICA LOMELI CAZARES</t>
+  </si>
+  <si>
+    <t>SOFIA CAMPILLO VASCONCELOS</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -218,6 +221,11 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -242,15 +250,43 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -585,7 +621,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B53"/>
+  <dimension ref="A1:B54"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -1012,7 +1048,23 @@
         <v>53</v>
       </c>
     </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A54" s="3">
+        <v>116883</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
   </sheetData>
+  <conditionalFormatting sqref="A54">
+    <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
+      <formula>$S54=1</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="0" priority="2" stopIfTrue="1">
+      <formula>$S53=1</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError sqref="A1:B1" numberStoredAsText="1"/>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-04-29 09:26)
</commit_message>
<xml_diff>
--- a/administrador/directorio_asesores.xlsx
+++ b/administrador/directorio_asesores.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02F7E6AB-177F-F349-97C0-2F6D0D2240A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A30E5F01-E3FA-7041-A56A-6FE24C036A79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
   <si>
     <t>Clave</t>
   </si>
@@ -198,13 +198,22 @@
   </si>
   <si>
     <t>SOFIA CAMPILLO VASCONCELOS</t>
+  </si>
+  <si>
+    <t>GERARDO DANIEL BARAJAS TORRES</t>
+  </si>
+  <si>
+    <t>MARIO IVAN ROMERO GONZALEZ</t>
+  </si>
+  <si>
+    <t>MONSERRAT VELASCO SANTOS</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -229,6 +238,12 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -250,7 +265,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -258,6 +273,7 @@
       <alignment vertical="center"/>
       <protection hidden="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -621,7 +637,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B54"/>
+  <dimension ref="A1:B57"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -1054,6 +1070,30 @@
       </c>
       <c r="B54" s="2" t="s">
         <v>54</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A55" s="4">
+        <v>117440</v>
+      </c>
+      <c r="B55" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A56" s="4">
+        <v>118069</v>
+      </c>
+      <c r="B56" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A57" s="4">
+        <v>16795</v>
+      </c>
+      <c r="B57" t="s">
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-04-29 09:29)
</commit_message>
<xml_diff>
--- a/administrador/directorio_asesores.xlsx
+++ b/administrador/directorio_asesores.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A30E5F01-E3FA-7041-A56A-6FE24C036A79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDE84FE3-C2BC-0B46-836F-72EBBB306764}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1090,7 +1090,7 @@
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A57" s="4">
-        <v>16795</v>
+        <v>116795</v>
       </c>
       <c r="B57" t="s">
         <v>55</v>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-05-06 15:21)
</commit_message>
<xml_diff>
--- a/administrador/directorio_asesores.xlsx
+++ b/administrador/directorio_asesores.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A7C89EC-A3C0-1A46-8994-ABC58FF78A39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29A883AB-9662-FD44-AD07-ADC2BDCE398C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2760" yWindow="3160" windowWidth="24460" windowHeight="16320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Directorio" sheetId="1" r:id="rId1"/>
@@ -262,10 +262,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -274,11 +275,45 @@
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{A33D40C2-E868-5147-918D-4D86DB7D513E}"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="4">
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <border>
         <top style="thin">
@@ -637,7 +672,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B57"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -896,7 +931,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>108920</v>
       </c>
@@ -904,7 +939,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>109007</v>
       </c>
@@ -912,7 +947,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>109819</v>
       </c>
@@ -920,7 +955,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>109998</v>
       </c>
@@ -928,7 +963,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>110105</v>
       </c>
@@ -936,7 +971,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>110453</v>
       </c>
@@ -944,7 +979,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>110575</v>
       </c>
@@ -952,7 +987,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>111056</v>
       </c>
@@ -960,7 +995,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>111960</v>
       </c>
@@ -968,7 +1003,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>112083</v>
       </c>
@@ -976,7 +1011,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>112522</v>
       </c>
@@ -984,7 +1019,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>113076</v>
       </c>
@@ -992,7 +1027,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>113450</v>
       </c>
@@ -1000,7 +1035,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>114100</v>
       </c>
@@ -1008,7 +1043,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>114157</v>
       </c>
@@ -1016,13 +1051,14 @@
         <v>47</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>114431</v>
       </c>
       <c r="B48" t="s">
         <v>48</v>
       </c>
+      <c r="G48" s="5"/>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A49">
@@ -1098,11 +1134,16 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A54">
-    <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
+    <cfRule type="expression" dxfId="3" priority="3" stopIfTrue="1">
       <formula>$S54=1</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="2" stopIfTrue="1">
+    <cfRule type="expression" dxfId="2" priority="4" stopIfTrue="1">
       <formula>$S53=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G48">
+    <cfRule type="expression" dxfId="0" priority="1" stopIfTrue="1">
+      <formula>$B48&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-06-04 11:59)
</commit_message>
<xml_diff>
--- a/administrador/directorio_asesores.xlsx
+++ b/administrador/directorio_asesores.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29A883AB-9662-FD44-AD07-ADC2BDCE398C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A761E66A-D66B-7043-BE04-455C9D822657}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2760" yWindow="3160" windowWidth="24460" windowHeight="16320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Directorio" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="51">
   <si>
     <t>Clave</t>
   </si>
@@ -53,9 +53,6 @@
     <t>MARIA FERNANDA CARLOS VAZQUEZ</t>
   </si>
   <si>
-    <t>ALEJANDRA GABRIELA AMBRIZ GOMEZ</t>
-  </si>
-  <si>
     <t>PAULINA RODRIGUEZ DE LA MORA</t>
   </si>
   <si>
@@ -71,9 +68,6 @@
     <t>KAREN MUÐOZ GARCIA</t>
   </si>
   <si>
-    <t>ALEJANDRA IVETTE PEDROZA MACIAS</t>
-  </si>
-  <si>
     <t>MONICA ANDREA AMBRIZ GOMEZ</t>
   </si>
   <si>
@@ -89,9 +83,6 @@
     <t>MARIA TERESA ASENCIO LOZANO</t>
   </si>
   <si>
-    <t>JOSE ALBERTO CORONADO ROSAS</t>
-  </si>
-  <si>
     <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
   </si>
   <si>
@@ -134,18 +125,9 @@
     <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
   </si>
   <si>
-    <t>ROCIO IVON RUIZ GARCIA</t>
-  </si>
-  <si>
-    <t>ANGELICA YADIRA ROMERO JAUREGUI</t>
-  </si>
-  <si>
     <t>ISAI ANTONIO ROJAS MARTINEZ</t>
   </si>
   <si>
-    <t>MIRIAM ROCIO LOMELI CHAVEZ</t>
-  </si>
-  <si>
     <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
   </si>
   <si>
@@ -158,18 +140,12 @@
     <t>JORGE ANTONIO LUNA LARA</t>
   </si>
   <si>
-    <t>CLAUDIA VALERIA HERNANDEZ MACIAS</t>
-  </si>
-  <si>
     <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
   </si>
   <si>
     <t>LAURA DOLORES MONTAÐO MONTAÐO</t>
   </si>
   <si>
-    <t>BRUNO BRAULIO MACIAS ALVAREZ</t>
-  </si>
-  <si>
     <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
   </si>
   <si>
@@ -207,6 +183,9 @@
   </si>
   <si>
     <t>MONSERRAT VELASCO SANTOS</t>
+  </si>
+  <si>
+    <t>FECHA_CONEXION</t>
   </si>
 </sst>
 </file>
@@ -266,7 +245,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -276,12 +255,21 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{A33D40C2-E868-5147-918D-4D86DB7D513E}"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="7">
     <dxf>
       <border>
         <left style="hair">
@@ -297,6 +285,47 @@
           <color indexed="64"/>
         </bottom>
       </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
     </dxf>
     <dxf>
       <border>
@@ -675,356 +704,488 @@
   <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2">
+      <c r="C1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" s="6">
+        <v>100677</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="8">
+        <v>44999</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" s="6">
+        <v>101640</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="8">
+        <v>45104</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" s="6">
+        <v>102825</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="8">
+        <v>45117</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" s="6">
+        <v>103982</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="8">
+        <v>45216</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" s="6">
+        <v>104343</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="8">
+        <v>45201</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" s="6">
+        <v>104718</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="8">
+        <v>45264</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" s="6">
+        <v>104750</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="8">
+        <v>45236</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" s="6">
+        <v>105696</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" s="8">
+        <v>45279</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" s="6">
+        <v>106018</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" s="8">
+        <v>45344</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11" s="6">
+        <v>107488</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" s="8">
+        <v>45440</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" s="6">
+        <v>108404</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" s="8">
+        <v>45467</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" s="6">
+        <v>108405</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" s="8">
+        <v>45471</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14" s="6">
+        <v>109007</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C14" s="8">
+        <v>45525</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15" s="6">
+        <v>109998</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C15" s="8">
+        <v>45596</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A16" s="6">
+        <v>110105</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" s="8">
+        <v>45560</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17" s="6">
+        <v>110453</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C17" s="8">
+        <v>45600</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18" s="6">
+        <v>110575</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C18" s="8">
+        <v>45583</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" s="6">
+        <v>111056</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C19" s="8">
+        <v>45639</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20" s="6">
+        <v>112083</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C20" s="8">
+        <v>45736</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A21" s="6">
+        <v>112522</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C21" s="8">
+        <v>45776</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A22" s="6">
+        <v>113450</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C22" s="8">
+        <v>45852</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A23" s="6">
+        <v>114100</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C23" s="8">
+        <v>45863</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A24" s="6">
+        <v>114157</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C24" s="8">
+        <v>45904</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A25" s="6">
+        <v>115047</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C25" s="8">
+        <v>45944</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A26" s="6">
+        <v>115404</v>
+      </c>
+      <c r="B26" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="C26" s="8">
+        <v>45986</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A27" s="6">
+        <v>116876</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="C27" s="8">
+        <v>46111</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A28" s="6">
+        <v>116883</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="C28" s="8">
+        <v>46126</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A29" s="6">
+        <v>117440</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C29" s="8">
+        <v>46149</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A30" s="6">
         <v>47116</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B30" s="7" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3">
+      <c r="C30" s="8">
+        <v>44616</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A31" s="6">
         <v>59120</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B31" s="7" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4">
+      <c r="C31" s="8">
+        <v>44708</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A32" s="6">
         <v>63441</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B32" s="7" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5">
-        <v>64502</v>
-      </c>
-      <c r="B5" t="s">
+      <c r="C32" s="8">
+        <v>44733</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A33" s="6">
+        <v>65046</v>
+      </c>
+      <c r="B33" s="7" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6">
-        <v>65046</v>
-      </c>
-      <c r="B6" t="s">
+      <c r="C33" s="8">
+        <v>44763</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A34" s="6">
+        <v>69684</v>
+      </c>
+      <c r="B34" s="7" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7">
-        <v>69684</v>
-      </c>
-      <c r="B7" t="s">
+      <c r="C34" s="8">
+        <v>44771</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A35" s="6">
+        <v>80122</v>
+      </c>
+      <c r="B35" s="7" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8">
-        <v>80122</v>
-      </c>
-      <c r="B8" t="s">
+      <c r="C35" s="8">
+        <v>43371</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A36" s="6">
+        <v>80925</v>
+      </c>
+      <c r="B36" s="7" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A9">
-        <v>80925</v>
-      </c>
-      <c r="B9" t="s">
+      <c r="C36" s="8">
+        <v>43439</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A37" s="6">
+        <v>81044</v>
+      </c>
+      <c r="B37" s="7" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A10">
-        <v>81044</v>
-      </c>
-      <c r="B10" t="s">
+      <c r="C37" s="8">
+        <v>44872</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A38" s="6">
+        <v>87538</v>
+      </c>
+      <c r="B38" s="7" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A11">
-        <v>81618</v>
-      </c>
-      <c r="B11" t="s">
+      <c r="C38" s="8">
+        <v>43731</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A39" s="6">
+        <v>88234</v>
+      </c>
+      <c r="B39" s="7" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A12">
-        <v>87538</v>
-      </c>
-      <c r="B12" t="s">
+      <c r="C39" s="8">
+        <v>43794</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A40" s="6">
+        <v>90177</v>
+      </c>
+      <c r="B40" s="7" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A13">
-        <v>88234</v>
-      </c>
-      <c r="B13" t="s">
+      <c r="C40" s="8">
+        <v>43949</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A41" s="6">
+        <v>90355</v>
+      </c>
+      <c r="B41" s="7" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A14">
-        <v>90177</v>
-      </c>
-      <c r="B14" t="s">
+      <c r="C41" s="8">
+        <v>43949</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A42" s="6">
+        <v>94156</v>
+      </c>
+      <c r="B42" s="7" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A15">
-        <v>90355</v>
-      </c>
-      <c r="B15" t="s">
+      <c r="C42" s="8">
+        <v>44159</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A43" s="6">
+        <v>95148</v>
+      </c>
+      <c r="B43" s="7" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A16">
-        <v>94156</v>
-      </c>
-      <c r="B16" t="s">
+      <c r="C43" s="8">
+        <v>44916</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A44" s="6">
+        <v>98797</v>
+      </c>
+      <c r="B44" s="7" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A17">
-        <v>94205</v>
-      </c>
-      <c r="B17" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A18">
-        <v>95148</v>
-      </c>
-      <c r="B18" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A19">
-        <v>98797</v>
-      </c>
-      <c r="B19" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A20">
-        <v>100677</v>
-      </c>
-      <c r="B20" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A21">
-        <v>101640</v>
-      </c>
-      <c r="B21" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A22">
-        <v>102825</v>
-      </c>
-      <c r="B22" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A23">
-        <v>103982</v>
-      </c>
-      <c r="B23" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A24">
-        <v>104343</v>
-      </c>
-      <c r="B24" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A25">
-        <v>104718</v>
-      </c>
-      <c r="B25" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A26">
-        <v>104750</v>
-      </c>
-      <c r="B26" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A27">
-        <v>105696</v>
-      </c>
-      <c r="B27" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A28">
-        <v>106018</v>
-      </c>
-      <c r="B28" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A29">
-        <v>107488</v>
-      </c>
-      <c r="B29" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A30">
-        <v>108404</v>
-      </c>
-      <c r="B30" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A31">
-        <v>108405</v>
-      </c>
-      <c r="B31" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A32">
-        <v>108658</v>
-      </c>
-      <c r="B32" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A33">
-        <v>108920</v>
-      </c>
-      <c r="B33" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A34">
-        <v>109007</v>
-      </c>
-      <c r="B34" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A35">
-        <v>109819</v>
-      </c>
-      <c r="B35" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A36">
-        <v>109998</v>
-      </c>
-      <c r="B36" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A37">
-        <v>110105</v>
-      </c>
-      <c r="B37" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A38">
-        <v>110453</v>
-      </c>
-      <c r="B38" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A39">
-        <v>110575</v>
-      </c>
-      <c r="B39" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A40">
-        <v>111056</v>
-      </c>
-      <c r="B40" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A41">
-        <v>111960</v>
-      </c>
-      <c r="B41" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A42">
-        <v>112083</v>
-      </c>
-      <c r="B42" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A43">
-        <v>112522</v>
-      </c>
-      <c r="B43" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A44">
-        <v>113076</v>
-      </c>
-      <c r="B44" t="s">
-        <v>44</v>
+      <c r="C44" s="8">
+        <v>44342</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.2">
@@ -1032,7 +1193,7 @@
         <v>113450</v>
       </c>
       <c r="B45" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.2">
@@ -1040,7 +1201,7 @@
         <v>114100</v>
       </c>
       <c r="B46" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.2">
@@ -1048,7 +1209,7 @@
         <v>114157</v>
       </c>
       <c r="B47" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.2">
@@ -1056,7 +1217,7 @@
         <v>114431</v>
       </c>
       <c r="B48" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="G48" s="5"/>
     </row>
@@ -1065,7 +1226,7 @@
         <v>114664</v>
       </c>
       <c r="B49" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.2">
@@ -1073,7 +1234,7 @@
         <v>115047</v>
       </c>
       <c r="B50" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.2">
@@ -1081,7 +1242,7 @@
         <v>115404</v>
       </c>
       <c r="B51" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.2">
@@ -1089,7 +1250,7 @@
         <v>116060</v>
       </c>
       <c r="B52" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.2">
@@ -1097,7 +1258,7 @@
         <v>116876</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.2">
@@ -1105,7 +1266,7 @@
         <v>116883</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.2">
@@ -1113,7 +1274,7 @@
         <v>117440</v>
       </c>
       <c r="B55" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.2">
@@ -1121,7 +1282,7 @@
         <v>118069</v>
       </c>
       <c r="B56" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.2">
@@ -1129,21 +1290,41 @@
         <v>116795</v>
       </c>
       <c r="B57" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A54">
-    <cfRule type="expression" dxfId="3" priority="3" stopIfTrue="1">
+    <cfRule type="expression" dxfId="6" priority="7" stopIfTrue="1">
       <formula>$S54=1</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="4" stopIfTrue="1">
+    <cfRule type="expression" dxfId="5" priority="8" stopIfTrue="1">
       <formula>$S53=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G48">
+    <cfRule type="expression" dxfId="4" priority="5" stopIfTrue="1">
+      <formula>$B48&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2:C44">
+    <cfRule type="expression" dxfId="3" priority="4" stopIfTrue="1">
+      <formula>+#REF!="p"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2:A44">
+    <cfRule type="expression" dxfId="2" priority="3" stopIfTrue="1">
+      <formula>$B2&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B2:B44">
+    <cfRule type="expression" dxfId="1" priority="2" stopIfTrue="1">
+      <formula>$B2&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C2:C44">
     <cfRule type="expression" dxfId="0" priority="1" stopIfTrue="1">
-      <formula>$B48&lt;&gt;""</formula>
+      <formula>$B2&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-07-07 21:02)
</commit_message>
<xml_diff>
--- a/administrador/directorio_asesores.xlsx
+++ b/administrador/directorio_asesores.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10413"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A761E66A-D66B-7043-BE04-455C9D822657}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90E2918B-BB1F-EC48-8CDC-9A1536889D65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4340" yWindow="600" windowWidth="24460" windowHeight="16160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Directorio" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
   <si>
     <t>Clave</t>
   </si>
@@ -155,30 +155,18 @@
     <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
   </si>
   <si>
-    <t>MARIA JOSE GUZMAN ZAMORA</t>
-  </si>
-  <si>
-    <t>LINDA TANIA MIROSLAVA ENRIQUEZ PRECIADO</t>
-  </si>
-  <si>
     <t>VELIA PATRICIA BERNAL RAMOS</t>
   </si>
   <si>
     <t>ANA VERONICA GONZALEZ GAYTAN</t>
   </si>
   <si>
-    <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
-  </si>
-  <si>
     <t>PAULA ANGELICA LOMELI CAZARES</t>
   </si>
   <si>
     <t>SOFIA CAMPILLO VASCONCELOS</t>
   </si>
   <si>
-    <t>GERARDO DANIEL BARAJAS TORRES</t>
-  </si>
-  <si>
     <t>MARIO IVAN ROMERO GONZALEZ</t>
   </si>
   <si>
@@ -186,13 +174,19 @@
   </si>
   <si>
     <t>FECHA_CONEXION</t>
+  </si>
+  <si>
+    <t>ALEJANDRA GABRIELA AMBRIZ GOMEZ</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy;@"/>
+  </numFmts>
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -220,6 +214,11 @@
     <font>
       <sz val="10"/>
       <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -255,50 +254,36 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
     </xf>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{A33D40C2-E868-5147-918D-4D86DB7D513E}"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="6">
     <dxf>
       <border>
-        <left style="hair">
-          <color indexed="64"/>
+        <left style="thin">
+          <color theme="0" tint="-0.14996795556505021"/>
         </left>
-        <right style="hair">
-          <color indexed="64"/>
+        <right style="thin">
+          <color theme="0" tint="-0.14996795556505021"/>
         </right>
-        <top style="hair">
-          <color indexed="64"/>
+        <top style="thin">
+          <color theme="0" tint="-0.14996795556505021"/>
         </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
+        <bottom style="thin">
+          <color theme="0" tint="-0.14996795556505021"/>
         </bottom>
       </border>
     </dxf>
@@ -712,73 +697,73 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" s="6">
-        <v>100677</v>
+        <v>87538</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="C2" s="8">
-        <v>44999</v>
+        <v>43731</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="6">
-        <v>101640</v>
+        <v>110453</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="C3" s="8">
-        <v>45104</v>
+        <v>45600</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="6">
-        <v>102825</v>
+        <v>80122</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="C4" s="8">
-        <v>45117</v>
+        <v>43371</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="6">
-        <v>103982</v>
+        <v>90355</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="C5" s="8">
-        <v>45216</v>
+        <v>43949</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="6">
-        <v>104343</v>
+        <v>47116</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>22</v>
+        <v>3</v>
       </c>
       <c r="C6" s="8">
-        <v>45201</v>
+        <v>44616</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="6">
-        <v>104718</v>
+        <v>111056</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="C7" s="8">
-        <v>45264</v>
+        <v>45639</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
@@ -794,535 +779,457 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="6">
-        <v>105696</v>
+        <v>94156</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="C9" s="8">
-        <v>45279</v>
+        <v>44159</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="6">
-        <v>106018</v>
+        <v>116883</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>26</v>
+        <v>43</v>
       </c>
       <c r="C10" s="8">
-        <v>45344</v>
+        <v>46126</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="6">
-        <v>107488</v>
+        <v>117440</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="C11" s="8">
-        <v>45440</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" s="6">
-        <v>108404</v>
+        <v>80925</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="C12" s="8">
-        <v>45467</v>
+        <v>43439</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="6">
-        <v>108405</v>
+        <v>105696</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C13" s="8">
-        <v>45471</v>
+        <v>45279</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="6">
-        <v>109007</v>
+        <v>103982</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="C14" s="8">
-        <v>45525</v>
+        <v>45216</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="6">
-        <v>109998</v>
+        <v>113450</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="C15" s="8">
-        <v>45596</v>
+        <v>45852</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="6">
-        <v>110105</v>
+        <v>110575</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C16" s="8">
-        <v>45560</v>
+        <v>45583</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="6">
-        <v>110453</v>
+        <v>116876</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>2</v>
+        <v>42</v>
       </c>
       <c r="C17" s="8">
-        <v>45600</v>
+        <v>46111</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="6">
-        <v>110575</v>
+        <v>104718</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="C18" s="8">
-        <v>45583</v>
+        <v>45264</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="6">
-        <v>111056</v>
+        <v>118069</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="C19" s="8">
-        <v>45639</v>
+        <v>46192</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="6">
-        <v>112083</v>
+        <v>115047</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="C20" s="8">
-        <v>45736</v>
+        <v>45944</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="6">
-        <v>112522</v>
+        <v>100677</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="C21" s="8">
-        <v>45776</v>
+        <v>44999</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="6">
-        <v>113450</v>
+        <v>107488</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="C22" s="8">
-        <v>45852</v>
+        <v>45440</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="6">
-        <v>114100</v>
+        <v>115404</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C23" s="8">
-        <v>45863</v>
+        <v>45986</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" s="6">
-        <v>114157</v>
+        <v>95148</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>39</v>
+        <v>16</v>
       </c>
       <c r="C24" s="8">
-        <v>45904</v>
+        <v>44916</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" s="6">
-        <v>115047</v>
+        <v>108404</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="C25" s="8">
-        <v>45944</v>
+        <v>45467</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" s="6">
-        <v>115404</v>
+        <v>88234</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="C26" s="8">
-        <v>45986</v>
+        <v>43794</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" s="6">
-        <v>116876</v>
+        <v>102825</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="C27" s="8">
-        <v>46111</v>
+        <v>45117</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" s="6">
-        <v>116883</v>
+        <v>104343</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="C28" s="8">
-        <v>46126</v>
+        <v>45201</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" s="6">
-        <v>117440</v>
+        <v>90177</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>49</v>
+        <v>13</v>
       </c>
       <c r="C29" s="8">
-        <v>46149</v>
+        <v>43949</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" s="6">
-        <v>47116</v>
+        <v>65046</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C30" s="8">
-        <v>44616</v>
+        <v>44763</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" s="6">
-        <v>59120</v>
+        <v>114100</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>4</v>
+        <v>38</v>
       </c>
       <c r="C31" s="8">
-        <v>44708</v>
+        <v>45863</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A32" s="6">
-        <v>63441</v>
+        <v>114157</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>5</v>
+        <v>39</v>
       </c>
       <c r="C32" s="8">
-        <v>44733</v>
+        <v>45904</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" s="6">
-        <v>65046</v>
+        <v>106018</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="C33" s="8">
-        <v>44763</v>
+        <v>45344</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" s="6">
-        <v>69684</v>
+        <v>108405</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>7</v>
+        <v>29</v>
       </c>
       <c r="C34" s="8">
-        <v>44771</v>
+        <v>45471</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" s="6">
-        <v>80122</v>
+        <v>110105</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="C35" s="8">
-        <v>43371</v>
+        <v>45560</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" s="6">
-        <v>80925</v>
+        <v>98797</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="C36" s="8">
-        <v>43439</v>
+        <v>44342</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" s="6">
-        <v>81044</v>
+        <v>112083</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="C37" s="8">
-        <v>44872</v>
+        <v>45736</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" s="6">
-        <v>87538</v>
+        <v>109007</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="C38" s="8">
-        <v>43731</v>
+        <v>45525</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" s="6">
-        <v>88234</v>
+        <v>101640</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="C39" s="8">
-        <v>43794</v>
+        <v>45104</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40" s="6">
-        <v>90177</v>
+        <v>64502</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>13</v>
+        <v>47</v>
       </c>
       <c r="C40" s="8">
-        <v>43949</v>
+        <v>42173</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" s="6">
-        <v>90355</v>
+        <v>63441</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="C41" s="8">
-        <v>43949</v>
+        <v>44733</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" s="6">
-        <v>94156</v>
+        <v>81044</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C42" s="8">
-        <v>44159</v>
+        <v>44872</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A43" s="6">
-        <v>95148</v>
+        <v>109998</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="C43" s="8">
-        <v>44916</v>
+        <v>45596</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A44" s="6">
-        <v>98797</v>
+        <v>69684</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="C44" s="8">
-        <v>44342</v>
+        <v>44771</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A45">
-        <v>113450</v>
-      </c>
-      <c r="B45" t="s">
-        <v>37</v>
+      <c r="A45" s="6">
+        <v>59120</v>
+      </c>
+      <c r="B45" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C45" s="8">
+        <v>44708</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A46">
-        <v>114100</v>
-      </c>
-      <c r="B46" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A47">
-        <v>114157</v>
-      </c>
-      <c r="B47" t="s">
-        <v>39</v>
+      <c r="A46" s="6">
+        <v>112522</v>
+      </c>
+      <c r="B46" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C46" s="8">
+        <v>45776</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A48">
-        <v>114431</v>
-      </c>
-      <c r="B48" t="s">
-        <v>40</v>
-      </c>
       <c r="G48" s="5"/>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A49">
-        <v>114664</v>
-      </c>
-      <c r="B49" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A50">
-        <v>115047</v>
-      </c>
-      <c r="B50" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A51">
-        <v>115404</v>
-      </c>
-      <c r="B51" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A52">
-        <v>116060</v>
-      </c>
-      <c r="B52" t="s">
-        <v>44</v>
-      </c>
-    </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A53" s="2">
-        <v>116876</v>
-      </c>
-      <c r="B53" s="1" t="s">
-        <v>45</v>
-      </c>
+      <c r="A53" s="2"/>
+      <c r="B53" s="1"/>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A54" s="3">
-        <v>116883</v>
-      </c>
-      <c r="B54" s="2" t="s">
-        <v>46</v>
-      </c>
+      <c r="A54" s="3"/>
+      <c r="B54" s="2"/>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A55" s="4">
-        <v>117440</v>
-      </c>
-      <c r="B55" t="s">
-        <v>49</v>
-      </c>
+      <c r="A55" s="4"/>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A56" s="4">
-        <v>118069</v>
-      </c>
-      <c r="B56" t="s">
-        <v>48</v>
-      </c>
+      <c r="A56" s="4"/>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A57" s="4">
-        <v>116795</v>
-      </c>
-      <c r="B57" t="s">
-        <v>47</v>
-      </c>
+      <c r="A57" s="4"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A54">
-    <cfRule type="expression" dxfId="6" priority="7" stopIfTrue="1">
+    <cfRule type="expression" dxfId="5" priority="8" stopIfTrue="1">
       <formula>$S54=1</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="8" stopIfTrue="1">
+    <cfRule type="expression" dxfId="4" priority="9" stopIfTrue="1">
       <formula>$S53=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G48">
-    <cfRule type="expression" dxfId="4" priority="5" stopIfTrue="1">
+    <cfRule type="expression" dxfId="1" priority="6" stopIfTrue="1">
       <formula>$B48&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:C44">
-    <cfRule type="expression" dxfId="3" priority="4" stopIfTrue="1">
-      <formula>+#REF!="p"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A2:A44">
-    <cfRule type="expression" dxfId="2" priority="3" stopIfTrue="1">
-      <formula>$B2&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B2:B44">
-    <cfRule type="expression" dxfId="1" priority="2" stopIfTrue="1">
-      <formula>$B2&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C44">
+  <conditionalFormatting sqref="A2:C46">
     <cfRule type="expression" dxfId="0" priority="1" stopIfTrue="1">
       <formula>$B2&lt;&gt;""</formula>
     </cfRule>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-07-09 11:44)
</commit_message>
<xml_diff>
--- a/administrador/directorio_asesores.xlsx
+++ b/administrador/directorio_asesores.xlsx
@@ -270,23 +270,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{A33D40C2-E868-5147-918D-4D86DB7D513E}"/>
   </cellStyles>
-  <dxfs count="6">
-    <dxf>
-      <border>
-        <left style="thin">
-          <color theme="0" tint="-0.14996795556505021"/>
-        </left>
-        <right style="thin">
-          <color theme="0" tint="-0.14996795556505021"/>
-        </right>
-        <top style="thin">
-          <color theme="0" tint="-0.14996795556505021"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0" tint="-0.14996795556505021"/>
-        </bottom>
-      </border>
-    </dxf>
+  <dxfs count="4">
     <dxf>
       <border>
         <left style="hair">
@@ -304,27 +288,18 @@
       </border>
     </dxf>
     <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
       <border>
-        <left style="hair">
-          <color indexed="64"/>
+        <left style="thin">
+          <color theme="0" tint="-0.14996795556505021"/>
         </left>
-        <right style="hair">
-          <color indexed="64"/>
+        <right style="thin">
+          <color theme="0" tint="-0.14996795556505021"/>
         </right>
-        <top style="hair">
-          <color indexed="64"/>
+        <top style="thin">
+          <color theme="0" tint="-0.14996795556505021"/>
         </top>
-        <bottom style="hair">
-          <color indexed="64"/>
+        <bottom style="thin">
+          <color theme="0" tint="-0.14996795556505021"/>
         </bottom>
       </border>
     </dxf>
@@ -1217,21 +1192,21 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A54">
-    <cfRule type="expression" dxfId="5" priority="8" stopIfTrue="1">
+    <cfRule type="expression" dxfId="3" priority="8" stopIfTrue="1">
       <formula>$S54=1</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="9" stopIfTrue="1">
+    <cfRule type="expression" dxfId="2" priority="9" stopIfTrue="1">
       <formula>$S53=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G48">
-    <cfRule type="expression" dxfId="1" priority="6" stopIfTrue="1">
-      <formula>$B48&lt;&gt;""</formula>
+  <conditionalFormatting sqref="A2:C46">
+    <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
+      <formula>$B2&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:C46">
-    <cfRule type="expression" dxfId="0" priority="1" stopIfTrue="1">
-      <formula>$B2&lt;&gt;""</formula>
+  <conditionalFormatting sqref="G48">
+    <cfRule type="expression" dxfId="0" priority="6" stopIfTrue="1">
+      <formula>$B48&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-07-10 16:56)
</commit_message>
<xml_diff>
--- a/administrador/directorio_asesores.xlsx
+++ b/administrador/directorio_asesores.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90E2918B-BB1F-EC48-8CDC-9A1536889D65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{903B84CC-ADD6-A34A-A88E-4DC396DF3CCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="600" windowWidth="24460" windowHeight="16160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Directorio" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Directorio!$A$1:$C$1</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -677,79 +680,79 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" s="6">
-        <v>87538</v>
+        <v>64502</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>11</v>
+        <v>47</v>
       </c>
       <c r="C2" s="8">
-        <v>43731</v>
+        <v>42173</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="6">
-        <v>110453</v>
+        <v>80122</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C3" s="8">
-        <v>45600</v>
+        <v>43371</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="6">
-        <v>80122</v>
+        <v>80925</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C4" s="8">
-        <v>43371</v>
+        <v>43439</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="6">
-        <v>90355</v>
+        <v>87538</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C5" s="8">
-        <v>43949</v>
+        <v>43731</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="6">
-        <v>47116</v>
+        <v>88234</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="C6" s="8">
-        <v>44616</v>
+        <v>43794</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="6">
-        <v>111056</v>
+        <v>90355</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="C7" s="8">
-        <v>45639</v>
+        <v>43949</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="6">
-        <v>104750</v>
+        <v>90177</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="C8" s="8">
-        <v>45236</v>
+        <v>43949</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
@@ -765,409 +768,409 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="6">
-        <v>116883</v>
+        <v>98797</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>43</v>
+        <v>17</v>
       </c>
       <c r="C10" s="8">
-        <v>46126</v>
+        <v>44342</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="6">
-        <v>117440</v>
+        <v>47116</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>45</v>
+        <v>3</v>
       </c>
       <c r="C11" s="8">
-        <v>46149</v>
+        <v>44616</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" s="6">
-        <v>80925</v>
+        <v>59120</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C12" s="8">
-        <v>43439</v>
+        <v>44708</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="6">
-        <v>105696</v>
+        <v>63441</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="C13" s="8">
-        <v>45279</v>
+        <v>44733</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="6">
-        <v>103982</v>
+        <v>65046</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="C14" s="8">
-        <v>45216</v>
+        <v>44763</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="6">
-        <v>113450</v>
+        <v>69684</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>37</v>
+        <v>7</v>
       </c>
       <c r="C15" s="8">
-        <v>45852</v>
+        <v>44771</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="6">
-        <v>110575</v>
+        <v>81044</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="C16" s="8">
-        <v>45583</v>
+        <v>44872</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="6">
-        <v>116876</v>
+        <v>95148</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="C17" s="8">
-        <v>46111</v>
+        <v>44916</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="6">
-        <v>104718</v>
+        <v>100677</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C18" s="8">
-        <v>45264</v>
+        <v>44999</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="6">
-        <v>118069</v>
+        <v>101640</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>44</v>
+        <v>19</v>
       </c>
       <c r="C19" s="8">
-        <v>46192</v>
+        <v>45104</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="6">
-        <v>115047</v>
+        <v>102825</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="C20" s="8">
-        <v>45944</v>
+        <v>45117</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="6">
-        <v>100677</v>
+        <v>104343</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C21" s="8">
-        <v>44999</v>
+        <v>45201</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="6">
-        <v>107488</v>
+        <v>103982</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="C22" s="8">
-        <v>45440</v>
+        <v>45216</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="6">
-        <v>115404</v>
+        <v>104750</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>41</v>
+        <v>24</v>
       </c>
       <c r="C23" s="8">
-        <v>45986</v>
+        <v>45236</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" s="6">
-        <v>95148</v>
+        <v>104718</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="C24" s="8">
-        <v>44916</v>
+        <v>45264</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" s="6">
-        <v>108404</v>
+        <v>105696</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C25" s="8">
-        <v>45467</v>
+        <v>45279</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" s="6">
-        <v>88234</v>
+        <v>106018</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="C26" s="8">
-        <v>43794</v>
+        <v>45344</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" s="6">
-        <v>102825</v>
+        <v>107488</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="C27" s="8">
-        <v>45117</v>
+        <v>45440</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" s="6">
-        <v>104343</v>
+        <v>108404</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="C28" s="8">
-        <v>45201</v>
+        <v>45467</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" s="6">
-        <v>90177</v>
+        <v>108405</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="C29" s="8">
-        <v>43949</v>
+        <v>45471</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" s="6">
-        <v>65046</v>
+        <v>109007</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="C30" s="8">
-        <v>44763</v>
+        <v>45525</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" s="6">
-        <v>114100</v>
+        <v>110105</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="C31" s="8">
-        <v>45863</v>
+        <v>45560</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A32" s="6">
-        <v>114157</v>
+        <v>110575</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="C32" s="8">
-        <v>45904</v>
+        <v>45583</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" s="6">
-        <v>106018</v>
+        <v>109998</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C33" s="8">
-        <v>45344</v>
+        <v>45596</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" s="6">
-        <v>108405</v>
+        <v>110453</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="C34" s="8">
-        <v>45471</v>
+        <v>45600</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" s="6">
-        <v>110105</v>
+        <v>111056</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C35" s="8">
-        <v>45560</v>
+        <v>45639</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" s="6">
-        <v>98797</v>
+        <v>112083</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>17</v>
+        <v>35</v>
       </c>
       <c r="C36" s="8">
-        <v>44342</v>
+        <v>45736</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" s="6">
-        <v>112083</v>
+        <v>112522</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C37" s="8">
-        <v>45736</v>
+        <v>45776</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" s="6">
-        <v>109007</v>
+        <v>113450</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="C38" s="8">
-        <v>45525</v>
+        <v>45852</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" s="6">
-        <v>101640</v>
+        <v>114100</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="C39" s="8">
-        <v>45104</v>
+        <v>45863</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40" s="6">
-        <v>64502</v>
+        <v>114157</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="C40" s="8">
-        <v>42173</v>
+        <v>45904</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" s="6">
-        <v>63441</v>
+        <v>115047</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>5</v>
+        <v>40</v>
       </c>
       <c r="C41" s="8">
-        <v>44733</v>
+        <v>45944</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" s="6">
-        <v>81044</v>
+        <v>115404</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>10</v>
+        <v>41</v>
       </c>
       <c r="C42" s="8">
-        <v>44872</v>
+        <v>45986</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A43" s="6">
-        <v>109998</v>
+        <v>116876</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="C43" s="8">
-        <v>45596</v>
+        <v>46111</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A44" s="6">
-        <v>69684</v>
+        <v>116883</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>7</v>
+        <v>43</v>
       </c>
       <c r="C44" s="8">
-        <v>44771</v>
+        <v>46126</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A45" s="6">
-        <v>59120</v>
+        <v>117440</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>4</v>
+        <v>45</v>
       </c>
       <c r="C45" s="8">
-        <v>44708</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A46" s="6">
-        <v>112522</v>
+        <v>118069</v>
       </c>
       <c r="B46" s="7" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="C46" s="8">
-        <v>45776</v>
+        <v>46192</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.2">
@@ -1191,6 +1194,11 @@
       <c r="A57" s="4"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:C1" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C46">
+      <sortCondition ref="C1:C46"/>
+    </sortState>
+  </autoFilter>
   <conditionalFormatting sqref="A54">
     <cfRule type="expression" dxfId="3" priority="8" stopIfTrue="1">
       <formula>$S54=1</formula>

</xml_diff>

<commit_message>
fix: normalize advisor string matching and clean 200 null response for campaign snapshot lookup
</commit_message>
<xml_diff>
--- a/administrador/directorio_asesores.xlsx
+++ b/administrador/directorio_asesores.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{903B84CC-ADD6-A34A-A88E-4DC396DF3CCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90C6FB55-2846-8D4C-BC66-81323A5B00C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4340" yWindow="600" windowWidth="24460" windowHeight="16160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4340" yWindow="600" windowWidth="24460" windowHeight="16140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Directorio" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Directorio!$A$1:$C$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Directorio!$A$1:$C$46</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -664,6 +664,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
@@ -678,7 +679,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2" s="6">
         <v>64502</v>
       </c>
@@ -689,7 +690,7 @@
         <v>42173</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A3" s="6">
         <v>80122</v>
       </c>
@@ -700,7 +701,7 @@
         <v>43371</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A4" s="6">
         <v>80925</v>
       </c>
@@ -711,7 +712,7 @@
         <v>43439</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5" s="6">
         <v>87538</v>
       </c>
@@ -722,7 +723,7 @@
         <v>43731</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6" s="6">
         <v>88234</v>
       </c>
@@ -733,7 +734,7 @@
         <v>43794</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" s="6">
         <v>90355</v>
       </c>
@@ -744,7 +745,7 @@
         <v>43949</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8" s="6">
         <v>90177</v>
       </c>
@@ -755,7 +756,7 @@
         <v>43949</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" s="6">
         <v>94156</v>
       </c>
@@ -766,7 +767,7 @@
         <v>44159</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10" s="6">
         <v>98797</v>
       </c>
@@ -777,7 +778,7 @@
         <v>44342</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A11" s="6">
         <v>47116</v>
       </c>
@@ -788,7 +789,7 @@
         <v>44616</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A12" s="6">
         <v>59120</v>
       </c>
@@ -799,7 +800,7 @@
         <v>44708</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A13" s="6">
         <v>63441</v>
       </c>
@@ -810,7 +811,7 @@
         <v>44733</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14" s="6">
         <v>65046</v>
       </c>
@@ -821,7 +822,7 @@
         <v>44763</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A15" s="6">
         <v>69684</v>
       </c>
@@ -832,7 +833,7 @@
         <v>44771</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A16" s="6">
         <v>81044</v>
       </c>
@@ -843,7 +844,7 @@
         <v>44872</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17" s="6">
         <v>95148</v>
       </c>
@@ -854,7 +855,7 @@
         <v>44916</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A18" s="6">
         <v>100677</v>
       </c>
@@ -865,7 +866,7 @@
         <v>44999</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19" s="6">
         <v>101640</v>
       </c>
@@ -876,7 +877,7 @@
         <v>45104</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20" s="6">
         <v>102825</v>
       </c>
@@ -887,7 +888,7 @@
         <v>45117</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A21" s="6">
         <v>104343</v>
       </c>
@@ -898,7 +899,7 @@
         <v>45201</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22" s="6">
         <v>103982</v>
       </c>
@@ -909,7 +910,7 @@
         <v>45216</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A23" s="6">
         <v>104750</v>
       </c>
@@ -920,7 +921,7 @@
         <v>45236</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A24" s="6">
         <v>104718</v>
       </c>
@@ -931,7 +932,7 @@
         <v>45264</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A25" s="6">
         <v>105696</v>
       </c>
@@ -942,7 +943,7 @@
         <v>45279</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26" s="6">
         <v>106018</v>
       </c>
@@ -953,7 +954,7 @@
         <v>45344</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27" s="6">
         <v>107488</v>
       </c>
@@ -964,7 +965,7 @@
         <v>45440</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A28" s="6">
         <v>108404</v>
       </c>
@@ -975,7 +976,7 @@
         <v>45467</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29" s="6">
         <v>108405</v>
       </c>
@@ -986,7 +987,7 @@
         <v>45471</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30" s="6">
         <v>109007</v>
       </c>
@@ -997,7 +998,7 @@
         <v>45525</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A31" s="6">
         <v>110105</v>
       </c>
@@ -1008,7 +1009,7 @@
         <v>45560</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32" s="6">
         <v>110575</v>
       </c>
@@ -1019,7 +1020,7 @@
         <v>45583</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A33" s="6">
         <v>109998</v>
       </c>
@@ -1030,7 +1031,7 @@
         <v>45596</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A34" s="6">
         <v>110453</v>
       </c>
@@ -1041,7 +1042,7 @@
         <v>45600</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A35" s="6">
         <v>111056</v>
       </c>
@@ -1052,7 +1053,7 @@
         <v>45639</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A36" s="6">
         <v>112083</v>
       </c>
@@ -1063,7 +1064,7 @@
         <v>45736</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A37" s="6">
         <v>112522</v>
       </c>
@@ -1074,7 +1075,7 @@
         <v>45776</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A38" s="6">
         <v>113450</v>
       </c>
@@ -1085,7 +1086,7 @@
         <v>45852</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A39" s="6">
         <v>114100</v>
       </c>
@@ -1107,7 +1108,7 @@
         <v>45904</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A41" s="6">
         <v>115047</v>
       </c>
@@ -1118,7 +1119,7 @@
         <v>45944</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A42" s="6">
         <v>115404</v>
       </c>
@@ -1129,7 +1130,7 @@
         <v>45986</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A43" s="6">
         <v>116876</v>
       </c>
@@ -1151,7 +1152,7 @@
         <v>46126</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A45" s="6">
         <v>117440</v>
       </c>
@@ -1162,7 +1163,7 @@
         <v>46149</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A46" s="6">
         <v>118069</v>
       </c>
@@ -1194,7 +1195,13 @@
       <c r="A57" s="4"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C1" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <autoFilter ref="A1:C46" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="HANA SOFIA LOPEZ QUIÐONEZ"/>
+        <filter val="SOFIA CAMPILLO VASCONCELOS"/>
+      </filters>
+    </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C46">
       <sortCondition ref="C1:C46"/>
     </sortState>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-08-17 12:13)
</commit_message>
<xml_diff>
--- a/administrador/directorio_asesores.xlsx
+++ b/administrador/directorio_asesores.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90C6FB55-2846-8D4C-BC66-81323A5B00C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2559803-5AC3-2F47-AB0D-BDA5F055940A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="600" windowWidth="24460" windowHeight="16140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
   <si>
     <t>Clave</t>
   </si>
@@ -180,6 +180,9 @@
   </si>
   <si>
     <t>ALEJANDRA GABRIELA AMBRIZ GOMEZ</t>
+  </si>
+  <si>
+    <t>JOSE ANTEMIO OLIVA SANTOS</t>
   </si>
 </sst>
 </file>
@@ -234,7 +237,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -242,12 +245,38 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -268,12 +297,91 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{A33D40C2-E868-5147-918D-4D86DB7D513E}"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="10">
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <border>
         <left style="hair">
@@ -664,7 +772,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
@@ -679,7 +786,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="2" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" s="6">
         <v>64502</v>
       </c>
@@ -690,7 +797,7 @@
         <v>42173</v>
       </c>
     </row>
-    <row r="3" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="6">
         <v>80122</v>
       </c>
@@ -701,7 +808,7 @@
         <v>43371</v>
       </c>
     </row>
-    <row r="4" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="6">
         <v>80925</v>
       </c>
@@ -712,7 +819,7 @@
         <v>43439</v>
       </c>
     </row>
-    <row r="5" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="6">
         <v>87538</v>
       </c>
@@ -723,7 +830,7 @@
         <v>43731</v>
       </c>
     </row>
-    <row r="6" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="6">
         <v>88234</v>
       </c>
@@ -734,7 +841,7 @@
         <v>43794</v>
       </c>
     </row>
-    <row r="7" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="6">
         <v>90355</v>
       </c>
@@ -745,7 +852,7 @@
         <v>43949</v>
       </c>
     </row>
-    <row r="8" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="6">
         <v>90177</v>
       </c>
@@ -756,7 +863,7 @@
         <v>43949</v>
       </c>
     </row>
-    <row r="9" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="6">
         <v>94156</v>
       </c>
@@ -767,7 +874,7 @@
         <v>44159</v>
       </c>
     </row>
-    <row r="10" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="6">
         <v>98797</v>
       </c>
@@ -778,7 +885,7 @@
         <v>44342</v>
       </c>
     </row>
-    <row r="11" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="6">
         <v>47116</v>
       </c>
@@ -789,7 +896,7 @@
         <v>44616</v>
       </c>
     </row>
-    <row r="12" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" s="6">
         <v>59120</v>
       </c>
@@ -800,7 +907,7 @@
         <v>44708</v>
       </c>
     </row>
-    <row r="13" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="6">
         <v>63441</v>
       </c>
@@ -811,7 +918,7 @@
         <v>44733</v>
       </c>
     </row>
-    <row r="14" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="6">
         <v>65046</v>
       </c>
@@ -822,7 +929,7 @@
         <v>44763</v>
       </c>
     </row>
-    <row r="15" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="6">
         <v>69684</v>
       </c>
@@ -833,7 +940,7 @@
         <v>44771</v>
       </c>
     </row>
-    <row r="16" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="6">
         <v>81044</v>
       </c>
@@ -844,7 +951,7 @@
         <v>44872</v>
       </c>
     </row>
-    <row r="17" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="6">
         <v>95148</v>
       </c>
@@ -855,7 +962,7 @@
         <v>44916</v>
       </c>
     </row>
-    <row r="18" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="6">
         <v>100677</v>
       </c>
@@ -866,7 +973,7 @@
         <v>44999</v>
       </c>
     </row>
-    <row r="19" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="6">
         <v>101640</v>
       </c>
@@ -877,7 +984,7 @@
         <v>45104</v>
       </c>
     </row>
-    <row r="20" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="6">
         <v>102825</v>
       </c>
@@ -888,7 +995,7 @@
         <v>45117</v>
       </c>
     </row>
-    <row r="21" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="6">
         <v>104343</v>
       </c>
@@ -899,7 +1006,7 @@
         <v>45201</v>
       </c>
     </row>
-    <row r="22" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="6">
         <v>103982</v>
       </c>
@@ -910,7 +1017,7 @@
         <v>45216</v>
       </c>
     </row>
-    <row r="23" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="6">
         <v>104750</v>
       </c>
@@ -921,7 +1028,7 @@
         <v>45236</v>
       </c>
     </row>
-    <row r="24" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" s="6">
         <v>104718</v>
       </c>
@@ -932,7 +1039,7 @@
         <v>45264</v>
       </c>
     </row>
-    <row r="25" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" s="6">
         <v>105696</v>
       </c>
@@ -943,7 +1050,7 @@
         <v>45279</v>
       </c>
     </row>
-    <row r="26" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" s="6">
         <v>106018</v>
       </c>
@@ -954,7 +1061,7 @@
         <v>45344</v>
       </c>
     </row>
-    <row r="27" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" s="6">
         <v>107488</v>
       </c>
@@ -965,7 +1072,7 @@
         <v>45440</v>
       </c>
     </row>
-    <row r="28" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" s="6">
         <v>108404</v>
       </c>
@@ -976,7 +1083,7 @@
         <v>45467</v>
       </c>
     </row>
-    <row r="29" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" s="6">
         <v>108405</v>
       </c>
@@ -987,7 +1094,7 @@
         <v>45471</v>
       </c>
     </row>
-    <row r="30" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" s="6">
         <v>109007</v>
       </c>
@@ -998,7 +1105,7 @@
         <v>45525</v>
       </c>
     </row>
-    <row r="31" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" s="6">
         <v>110105</v>
       </c>
@@ -1009,7 +1116,7 @@
         <v>45560</v>
       </c>
     </row>
-    <row r="32" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A32" s="6">
         <v>110575</v>
       </c>
@@ -1020,7 +1127,7 @@
         <v>45583</v>
       </c>
     </row>
-    <row r="33" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" s="6">
         <v>109998</v>
       </c>
@@ -1031,7 +1138,7 @@
         <v>45596</v>
       </c>
     </row>
-    <row r="34" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" s="6">
         <v>110453</v>
       </c>
@@ -1042,7 +1149,7 @@
         <v>45600</v>
       </c>
     </row>
-    <row r="35" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" s="6">
         <v>111056</v>
       </c>
@@ -1053,7 +1160,7 @@
         <v>45639</v>
       </c>
     </row>
-    <row r="36" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" s="6">
         <v>112083</v>
       </c>
@@ -1064,7 +1171,7 @@
         <v>45736</v>
       </c>
     </row>
-    <row r="37" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" s="6">
         <v>112522</v>
       </c>
@@ -1075,7 +1182,7 @@
         <v>45776</v>
       </c>
     </row>
-    <row r="38" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" s="6">
         <v>113450</v>
       </c>
@@ -1086,7 +1193,7 @@
         <v>45852</v>
       </c>
     </row>
-    <row r="39" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" s="6">
         <v>114100</v>
       </c>
@@ -1108,7 +1215,7 @@
         <v>45904</v>
       </c>
     </row>
-    <row r="41" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" s="6">
         <v>115047</v>
       </c>
@@ -1119,7 +1226,7 @@
         <v>45944</v>
       </c>
     </row>
-    <row r="42" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" s="6">
         <v>115404</v>
       </c>
@@ -1130,7 +1237,7 @@
         <v>45986</v>
       </c>
     </row>
-    <row r="43" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A43" s="6">
         <v>116876</v>
       </c>
@@ -1152,7 +1259,7 @@
         <v>46126</v>
       </c>
     </row>
-    <row r="45" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A45" s="6">
         <v>117440</v>
       </c>
@@ -1163,7 +1270,7 @@
         <v>46149</v>
       </c>
     </row>
-    <row r="46" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A46" s="6">
         <v>118069</v>
       </c>
@@ -1172,6 +1279,17 @@
       </c>
       <c r="C46" s="8">
         <v>46192</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A47" s="9">
+        <v>118246</v>
+      </c>
+      <c r="B47" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="C47" s="11">
+        <v>46239</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.2">
@@ -1196,32 +1314,50 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:C46" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="HANA SOFIA LOPEZ QUIÐONEZ"/>
-        <filter val="SOFIA CAMPILLO VASCONCELOS"/>
-      </filters>
-    </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C46">
       <sortCondition ref="C1:C46"/>
     </sortState>
   </autoFilter>
   <conditionalFormatting sqref="A54">
-    <cfRule type="expression" dxfId="3" priority="8" stopIfTrue="1">
+    <cfRule type="expression" dxfId="9" priority="14" stopIfTrue="1">
       <formula>$S54=1</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="9" stopIfTrue="1">
+    <cfRule type="expression" dxfId="8" priority="15" stopIfTrue="1">
       <formula>$S53=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:C46">
-    <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
+    <cfRule type="expression" dxfId="7" priority="7" stopIfTrue="1">
       <formula>$B2&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G48">
-    <cfRule type="expression" dxfId="0" priority="6" stopIfTrue="1">
+    <cfRule type="expression" dxfId="6" priority="12" stopIfTrue="1">
       <formula>$B48&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B47">
+    <cfRule type="expression" dxfId="5" priority="5" stopIfTrue="1">
+      <formula>$S47=1</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="4" priority="6" stopIfTrue="1">
+      <formula>$S46=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A47">
+    <cfRule type="expression" dxfId="3" priority="3" stopIfTrue="1">
+      <formula>$S47=1</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="4" stopIfTrue="1">
+      <formula>$S46=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C47">
+    <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
+      <formula>$S47=1</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="0" priority="2" stopIfTrue="1">
+      <formula>$S46=1</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-08-17 13:23)
</commit_message>
<xml_diff>
--- a/administrador/directorio_asesores.xlsx
+++ b/administrador/directorio_asesores.xlsx
@@ -312,14 +312,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{A33D40C2-E868-5147-918D-4D86DB7D513E}"/>
   </cellStyles>
-  <dxfs count="10">
-    <dxf>
-      <border>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
+  <dxfs count="8">
     <dxf>
       <border>
         <left style="hair">
@@ -341,45 +334,6 @@
         <top style="thin">
           <color indexed="64"/>
         </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -419,6 +373,29 @@
         <top style="thin">
           <color indexed="64"/>
         </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -1318,46 +1295,42 @@
       <sortCondition ref="C1:C46"/>
     </sortState>
   </autoFilter>
+  <conditionalFormatting sqref="A47">
+    <cfRule type="expression" dxfId="7" priority="3" stopIfTrue="1">
+      <formula>$S47=1</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A54">
-    <cfRule type="expression" dxfId="9" priority="14" stopIfTrue="1">
+    <cfRule type="expression" dxfId="6" priority="14" stopIfTrue="1">
       <formula>$S54=1</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="15" stopIfTrue="1">
+    <cfRule type="expression" dxfId="5" priority="15" stopIfTrue="1">
       <formula>$S53=1</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="A47:B47">
+    <cfRule type="expression" dxfId="4" priority="4" stopIfTrue="1">
+      <formula>$S46=1</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A2:C46">
-    <cfRule type="expression" dxfId="7" priority="7" stopIfTrue="1">
+    <cfRule type="expression" dxfId="3" priority="7" stopIfTrue="1">
       <formula>$B2&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G48">
-    <cfRule type="expression" dxfId="6" priority="12" stopIfTrue="1">
-      <formula>$B48&lt;&gt;""</formula>
+  <conditionalFormatting sqref="B47:C47">
+    <cfRule type="expression" dxfId="2" priority="1" stopIfTrue="1">
+      <formula>$S47=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B47">
-    <cfRule type="expression" dxfId="5" priority="5" stopIfTrue="1">
-      <formula>$S47=1</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="4" priority="6" stopIfTrue="1">
+  <conditionalFormatting sqref="C47">
+    <cfRule type="expression" dxfId="1" priority="2" stopIfTrue="1">
       <formula>$S46=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A47">
-    <cfRule type="expression" dxfId="3" priority="3" stopIfTrue="1">
-      <formula>$S47=1</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="2" priority="4" stopIfTrue="1">
-      <formula>$S46=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C47">
-    <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
-      <formula>$S47=1</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="0" priority="2" stopIfTrue="1">
-      <formula>$S46=1</formula>
+  <conditionalFormatting sqref="G48">
+    <cfRule type="expression" dxfId="0" priority="12" stopIfTrue="1">
+      <formula>$B48&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>